<commit_message>
completion of queueLL and minor changes effective programs
</commit_message>
<xml_diff>
--- a/DSA_9(CCL)/Test case template.xlsx
+++ b/DSA_9(CCL)/Test case template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\anandms\Data Structures\DSA 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2858824b3e8e580e/Attachments/Desktop/DSA/DSA_9(CCL)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F04E520F-7106-4D9E-ACFC-9926E2EE96F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{F04E520F-7106-4D9E-ACFC-9926E2EE96F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4BEEAAE-56F9-4760-95EA-59CB7C56AC0C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BABC2A12-2E1B-4014-A65D-613E2A9B232D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BABC2A12-2E1B-4014-A65D-613E2A9B232D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
   <si>
     <t>Project Name</t>
   </si>
@@ -126,6 +126,9 @@
   </si>
   <si>
     <t>Test cases</t>
+  </si>
+  <si>
+    <t>_002</t>
   </si>
 </sst>
 </file>
@@ -555,20 +558,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{821C9AA7-398B-4C08-951D-378825B8F1E7}">
   <dimension ref="A1:J22"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.44140625" customWidth="1"/>
-    <col min="2" max="2" width="26.109375" customWidth="1"/>
-    <col min="3" max="3" width="27.77734375" customWidth="1"/>
-    <col min="4" max="4" width="22.88671875" customWidth="1"/>
-    <col min="5" max="5" width="18.88671875" customWidth="1"/>
+    <col min="1" max="1" width="21.42578125" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" customWidth="1"/>
+    <col min="4" max="4" width="22.85546875" customWidth="1"/>
+    <col min="5" max="5" width="18.85546875" customWidth="1"/>
     <col min="6" max="6" width="24" customWidth="1"/>
-    <col min="7" max="7" width="16.109375" customWidth="1"/>
+    <col min="7" max="7" width="16.140625" customWidth="1"/>
     <col min="8" max="9" width="17" customWidth="1"/>
-    <col min="10" max="10" width="11.5546875" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="25.8" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:10" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>29</v>
@@ -582,7 +585,7 @@
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -594,7 +597,7 @@
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -610,7 +613,7 @@
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -626,7 +629,7 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
@@ -642,7 +645,7 @@
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
@@ -658,7 +661,7 @@
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
@@ -672,7 +675,7 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>9</v>
       </c>
@@ -686,7 +689,7 @@
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -698,7 +701,7 @@
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>10</v>
       </c>
@@ -730,7 +733,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>20</v>
       </c>
@@ -762,8 +765,10 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="7"/>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
@@ -774,7 +779,7 @@
       <c r="I12" s="7"/>
       <c r="J12" s="7"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -786,7 +791,7 @@
       <c r="I13" s="4"/>
       <c r="J13" s="4"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="7"/>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
@@ -798,7 +803,7 @@
       <c r="I14" s="7"/>
       <c r="J14" s="7"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -810,7 +815,7 @@
       <c r="I15" s="4"/>
       <c r="J15" s="4"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="7"/>
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
@@ -822,7 +827,7 @@
       <c r="I16" s="7"/>
       <c r="J16" s="7"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="4"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -834,7 +839,7 @@
       <c r="I17" s="4"/>
       <c r="J17" s="4"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="7"/>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
@@ -846,7 +851,7 @@
       <c r="I18" s="7"/>
       <c r="J18" s="7"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="4"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -858,7 +863,7 @@
       <c r="I19" s="4"/>
       <c r="J19" s="4"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="7"/>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -870,7 +875,7 @@
       <c r="I20" s="7"/>
       <c r="J20" s="7"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="4"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -882,7 +887,7 @@
       <c r="I21" s="4"/>
       <c r="J21" s="4"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="7"/>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>

</xml_diff>